<commit_message>
Cursor: Apply local changes for cloud agent
</commit_message>
<xml_diff>
--- a/琐碎记录/赵孟頫故居一日游.xlsx
+++ b/琐碎记录/赵孟頫故居一日游.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="12780" activeTab="1"/>
+    <workbookView windowWidth="30720" windowHeight="12780" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="交通对比" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="254">
   <si>
     <t>路线</t>
   </si>
@@ -132,6 +132,12 @@
     <t>可省钱但耗时</t>
   </si>
   <si>
+    <t>精简版｜约8.5小时（08:00出门→16:30到家）｜只留故居+午饭+莲花庄，无加项</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>时间</t>
   </si>
   <si>
@@ -141,94 +147,172 @@
     <t>说明</t>
   </si>
   <si>
-    <t>07:20</t>
+    <t>08:00</t>
   </si>
   <si>
     <t>出发</t>
   </si>
   <si>
-    <t>古墩路站坐3号线往吴山前村，直达火车西站</t>
-  </si>
-  <si>
-    <t>07:50</t>
-  </si>
-  <si>
-    <t>杭州西站进站</t>
-  </si>
-  <si>
-    <t>安检、找检票口；西站站厅较大，留足时间</t>
-  </si>
-  <si>
-    <t>08:20前后</t>
+    <t>古墩路站3号线往吴山前村→火车西站，约30分钟</t>
+  </si>
+  <si>
+    <t>08:30</t>
+  </si>
+  <si>
+    <t>西站进站</t>
+  </si>
+  <si>
+    <t>安检候车约25–30分钟</t>
+  </si>
+  <si>
+    <t>09:00前后</t>
   </si>
   <si>
     <t>高铁去湖州</t>
   </si>
   <si>
-    <t>杭州西→湖州站，约22分钟（可选07:57、08:22附近车次，以当天时刻表为准）</t>
-  </si>
-  <si>
-    <t>08:50</t>
+    <t>杭州西→湖州站约22分钟；车次以12306为准</t>
+  </si>
+  <si>
+    <t>09:25</t>
   </si>
   <si>
     <t>到湖州站</t>
   </si>
   <si>
-    <t>打车约20-30分钟到故居；公交42路等到莲花庄约40分钟</t>
-  </si>
-  <si>
-    <t>09:30-11:30</t>
+    <t>打车约25分钟到故居/莲花庄一带</t>
+  </si>
+  <si>
+    <t>09:50-11:10</t>
   </si>
   <si>
     <t>赵孟頫故居</t>
   </si>
   <si>
-    <t>旧址纪念馆：生平陈列、松雪斋复原、书画刻石；认真看约1-1.5小时</t>
-  </si>
-  <si>
-    <t>11:30-13:00</t>
+    <t>约1小时20分；</t>
+  </si>
+  <si>
+    <t>11:10-12:20</t>
   </si>
   <si>
     <t>午饭</t>
   </si>
   <si>
-    <t>衣裳街/爱山广场一带：银鱼、湖羊、千张包、丁莲芳等</t>
-  </si>
-  <si>
-    <t>13:00-14:30</t>
+    <t>衣裳街约1小时；银鱼炒蛋等，少逛街</t>
+  </si>
+  <si>
+    <t>12:20-13:40</t>
   </si>
   <si>
     <t>莲花庄</t>
   </si>
   <si>
-    <t>赵孟頫别业；看莲花峰、松雪斋，与故居连成一线</t>
-  </si>
-  <si>
-    <t>14:30-15:30</t>
-  </si>
-  <si>
-    <t>可选加项</t>
-  </si>
-  <si>
-    <t>湖笔博物馆 / 飞英塔 / 潮音桥顺路，见「周边可选景点」表</t>
+    <t>约1小时20分逛园；不排飞英塔、湖笔馆</t>
+  </si>
+  <si>
+    <t>13:50</t>
+  </si>
+  <si>
+    <t>回湖州站</t>
+  </si>
+  <si>
+    <t>打车约25分钟</t>
+  </si>
+  <si>
+    <t>14:30前后</t>
+  </si>
+  <si>
+    <t>高铁回杭</t>
+  </si>
+  <si>
+    <t>湖州→杭州西约22分钟</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>到杭州西</t>
+  </si>
+  <si>
+    <t>3号线回古墩路约30分钟</t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>到家</t>
+  </si>
+  <si>
+    <t>合计约7.5小时；若车次错开，缓冲到16:30也仍在8.5小时内</t>
+  </si>
+  <si>
+    <t>—— 以下为标准版（约10小时，仍无「可选加项」）——</t>
+  </si>
+  <si>
+    <t>标准版｜约10小时（07:40出门→17:40到家）｜故居/午饭/莲花庄各多留一点</t>
+  </si>
+  <si>
+    <t>07:40</t>
+  </si>
+  <si>
+    <t>古墩路站3号线直达火车西站</t>
+  </si>
+  <si>
+    <t>08:10</t>
+  </si>
+  <si>
+    <t>安检候车</t>
+  </si>
+  <si>
+    <t>08:40前后</t>
+  </si>
+  <si>
+    <t>杭州西→湖州站约22分钟</t>
+  </si>
+  <si>
+    <t>09:05</t>
+  </si>
+  <si>
+    <t>09:30-11:00</t>
+  </si>
+  <si>
+    <t>约1.5小时；比精简版多半小时细看</t>
+  </si>
+  <si>
+    <t>11:00-12:30</t>
+  </si>
+  <si>
+    <t>衣裳街约1.5小时；可加一道整鱼（白鱼/鳜鱼）</t>
+  </si>
+  <si>
+    <t>12:30-14:20</t>
+  </si>
+  <si>
+    <t>约1小时50分；园内慢慢走，仍不去飞英塔</t>
+  </si>
+  <si>
+    <t>14:30</t>
+  </si>
+  <si>
+    <t>15:10前后</t>
   </si>
   <si>
     <t>15:40</t>
   </si>
   <si>
-    <t>回湖州站</t>
-  </si>
-  <si>
-    <t>打车赶16:30前后回杭州西的车；纪念馆16:00停止入馆</t>
-  </si>
-  <si>
-    <t>17:00左右</t>
-  </si>
-  <si>
-    <t>到杭州西</t>
-  </si>
-  <si>
-    <t>3号线原路回古墩路，约19:00前到家</t>
+    <t>3号线回古墩路</t>
+  </si>
+  <si>
+    <t>16:20</t>
+  </si>
+  <si>
+    <t>合计约8小时40分；车次若偏晚，到家可到17:40，仍≤10小时</t>
+  </si>
+  <si>
+    <t>时长核对</t>
+  </si>
+  <si>
+    <t>旧版出门到家约11–12小时（含可选加项+过长停留）。现精简约8.5小时、标准约10小时。往返交通约3.5–4小时；湖州停留精简约3.5小时、标准约4.5–5小时。</t>
   </si>
   <si>
     <t>类别</t>
@@ -273,7 +357,7 @@
     <t>莲花庄公园免费；周一仍可逛园但看不到故居展厅</t>
   </si>
   <si>
-    <t>预算(一人)</t>
+    <t>预算</t>
   </si>
   <si>
     <t>地铁往返</t>
@@ -288,10 +372,13 @@
     <t>约50-70元（以12306为准）</t>
   </si>
   <si>
+    <t>预算（多人打车）</t>
+  </si>
+  <si>
     <t>湖州打车两个来回</t>
   </si>
   <si>
-    <t>约60-100元（改公交可省）</t>
+    <t>约40-60元（改公交可省）</t>
   </si>
   <si>
     <t>约50-80元</t>
@@ -336,7 +423,7 @@
     <t>推荐路线</t>
   </si>
   <si>
-    <t>为何走西站</t>
+    <t>为啥走西站</t>
   </si>
   <si>
     <t>古墩路3号线直达杭州西；高铁约22分钟到湖州站</t>
@@ -537,9 +624,6 @@
     <t>时间怎么塞（参考）</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>核心线（已排入主表）</t>
   </si>
   <si>
@@ -676,9 +760,6 @@
   </si>
   <si>
     <t>秋季才主打；渔人码头一带餐馆常推</t>
-  </si>
-  <si>
-    <t>其他常见河鲜</t>
   </si>
   <si>
     <t>家常/馆子</t>
@@ -724,7 +805,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -742,6 +823,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF666666"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -891,7 +980,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -901,6 +990,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8F0E8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F0E6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8EEF5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1215,76 +1316,70 @@
     <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1293,10 +1388,10 @@
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1305,10 +1400,10 @@
     <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1317,10 +1412,10 @@
     <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1329,10 +1424,10 @@
     <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1341,19 +1436,35 @@
     <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1748,7 +1859,7 @@
     <col min="6" max="6" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:6">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1768,7 +1879,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" s="2" customFormat="1" ht="28.8" spans="1:6">
+    <row r="2" ht="28.8" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1788,7 +1899,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" s="2" customFormat="1" spans="1:6">
+    <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1808,7 +1919,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" s="2" customFormat="1" ht="28.8" spans="1:6">
+    <row r="4" ht="28.8" spans="1:6">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -1828,7 +1939,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" s="2" customFormat="1" spans="1:6">
+    <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
@@ -1848,7 +1959,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" s="2" customFormat="1" spans="1:6">
+    <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -1878,133 +1989,320 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="58" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="4" customFormat="1" ht="86.4" spans="1:3">
+      <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="1:3">
+      <c r="A2" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" s="2" customFormat="1" spans="1:3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" s="5" customFormat="1" spans="1:3">
+      <c r="A3" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="3" s="2" customFormat="1" spans="1:3">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="4" s="5" customFormat="1" spans="1:3">
+      <c r="A4" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="4" s="2" customFormat="1" ht="28.8" spans="1:3">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="2" t="s">
+    </row>
+    <row r="5" s="5" customFormat="1" spans="1:3">
+      <c r="A5" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="5" s="2" customFormat="1" spans="1:3">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="6" s="5" customFormat="1" spans="1:3">
+      <c r="A6" s="5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6" s="2" customFormat="1" ht="28.8" spans="1:3">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="2" t="s">
+    </row>
+    <row r="7" s="5" customFormat="1" spans="1:3">
+      <c r="A7" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" s="2" customFormat="1" spans="1:3">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="2" t="s">
+    </row>
+    <row r="8" s="5" customFormat="1" spans="1:3">
+      <c r="A8" s="5" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="8" s="2" customFormat="1" spans="1:3">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="9" s="5" customFormat="1" spans="1:3">
+      <c r="A9" s="5" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" s="2" customFormat="1" spans="1:3">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="2" t="s">
+    </row>
+    <row r="10" s="5" customFormat="1" spans="1:3">
+      <c r="A10" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="10" s="2" customFormat="1" spans="1:3">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="11" s="5" customFormat="1" spans="1:3">
+      <c r="A11" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="11" s="2" customFormat="1" spans="1:3">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="2" t="s">
+    </row>
+    <row r="12" s="5" customFormat="1" spans="1:3">
+      <c r="A12" s="5" t="s">
         <v>65</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" s="5" customFormat="1" spans="1:3">
+      <c r="A13" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" s="6" customFormat="1" spans="1:3">
+      <c r="A15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" s="7" customFormat="1" ht="72" spans="1:3">
+      <c r="A16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" s="1" customFormat="1" spans="1:3">
+      <c r="A17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" s="5" customFormat="1" spans="1:3">
+      <c r="A18" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" s="5" customFormat="1" spans="1:3">
+      <c r="A19" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" s="5" customFormat="1" spans="1:3">
+      <c r="A20" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" s="5" customFormat="1" spans="1:3">
+      <c r="A21" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" s="5" customFormat="1" spans="1:3">
+      <c r="A22" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" s="5" customFormat="1" spans="1:3">
+      <c r="A23" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" s="5" customFormat="1" spans="1:3">
+      <c r="A24" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" s="5" customFormat="1" spans="1:3">
+      <c r="A25" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" s="5" customFormat="1" spans="1:3">
+      <c r="A26" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" s="5" customFormat="1" spans="1:3">
+      <c r="A27" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" s="5" customFormat="1" spans="1:3">
+      <c r="A28" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="30" s="5" customFormat="1" ht="115.2" spans="1:3">
+      <c r="A30" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2020,196 +2318,196 @@
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="17.1111111111111" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" s="2" customFormat="1" spans="1:3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" s="2" customFormat="1" ht="28.8" spans="1:3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" ht="28.8" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" s="2" customFormat="1" spans="1:3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" s="2" customFormat="1" spans="1:3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" s="2" customFormat="1" spans="1:3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" s="2" customFormat="1" spans="1:3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" s="2" customFormat="1" spans="1:3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" s="2" customFormat="1" spans="1:3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" s="2" customFormat="1" spans="1:3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" s="2" customFormat="1" spans="1:3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" s="2" customFormat="1" spans="1:3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" s="2" customFormat="1" spans="1:3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" s="2" customFormat="1" spans="1:3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="2" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" s="2" customFormat="1" spans="1:3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="2" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="16" s="2" customFormat="1" spans="1:3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" s="2" customFormat="1" spans="1:3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="2" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2233,344 +2531,344 @@
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="1" ht="28.8" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>104</v>
+        <v>133</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="2" s="2" customFormat="1" spans="1:6">
-      <c r="A2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" s="2" customFormat="1" spans="1:6">
-      <c r="A3" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" s="2" customFormat="1" spans="1:6">
-      <c r="A4" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="5" s="2" customFormat="1" spans="1:6">
-      <c r="A5" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" s="2" customFormat="1" spans="1:6">
-      <c r="A6" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>133</v>
+        <v>162</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="7" s="2" customFormat="1" ht="28.8" spans="1:6">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" ht="28.8" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>135</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="9" ht="28.8" spans="1:6">
+      <c r="A9" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="8" s="2" customFormat="1" spans="1:6">
-      <c r="A8" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" s="2" customFormat="1" ht="28.8" spans="1:6">
-      <c r="A9" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" s="2" customFormat="1" spans="1:6">
-      <c r="A10" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" s="2" customFormat="1" ht="28.8" spans="1:6">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="11" ht="28.8" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>157</v>
+        <v>186</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>158</v>
+        <v>187</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="12" s="2" customFormat="1" spans="1:6">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>162</v>
+        <v>191</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>165</v>
+        <v>194</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>166</v>
+        <v>195</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" s="3" customFormat="1" spans="1:6">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
-        <v>167</v>
+        <v>196</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>169</v>
+        <v>197</v>
       </c>
       <c r="B15" t="s">
-        <v>170</v>
+        <v>198</v>
       </c>
       <c r="C15" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E15" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="F15" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>172</v>
+        <v>200</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>201</v>
       </c>
       <c r="C16" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E16" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="F16" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>175</v>
+        <v>203</v>
       </c>
       <c r="B17" t="s">
-        <v>176</v>
+        <v>204</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E17" t="s">
-        <v>177</v>
+        <v>205</v>
       </c>
       <c r="F17" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>178</v>
+        <v>206</v>
       </c>
       <c r="B18" t="s">
-        <v>179</v>
+        <v>207</v>
       </c>
       <c r="C18" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E18" t="s">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="F18" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2593,208 +2891,208 @@
     <col min="5" max="5" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:5">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>181</v>
+        <v>209</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>182</v>
+        <v>210</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>183</v>
+        <v>211</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>184</v>
+        <v>212</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" s="2" customFormat="1" ht="28.8" spans="1:5">
+    <row r="2" ht="28.8" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>185</v>
+        <v>213</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>186</v>
+        <v>214</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>187</v>
+        <v>215</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="3" s="2" customFormat="1" ht="28.8" spans="1:5">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" ht="28.8" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>191</v>
+        <v>219</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>192</v>
+        <v>220</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>193</v>
+        <v>221</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="4" s="2" customFormat="1" ht="28.8" spans="1:5">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" ht="28.8" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>196</v>
+        <v>224</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>197</v>
+        <v>225</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>198</v>
+        <v>226</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="5" s="2" customFormat="1" ht="28.8" spans="1:5">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" ht="28.8" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>200</v>
+        <v>228</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>201</v>
+        <v>229</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>202</v>
+        <v>230</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>203</v>
+        <v>231</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="6" s="2" customFormat="1" spans="1:5">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>233</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>206</v>
+        <v>234</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="7" s="2" customFormat="1" spans="1:5">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>211</v>
+        <v>239</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>212</v>
+        <v>240</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="8" s="2" customFormat="1" ht="28.8" spans="1:5">
-      <c r="A8" s="2" t="s">
-        <v>215</v>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="8" ht="28.8" spans="1:5">
+      <c r="A8" s="2">
+        <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>216</v>
+        <v>243</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>217</v>
+        <v>244</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>218</v>
+        <v>245</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="10" s="3" customFormat="1" spans="1:5">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>220</v>
+        <v>247</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>221</v>
+        <v>248</v>
       </c>
       <c r="B11" t="s">
-        <v>222</v>
+        <v>249</v>
       </c>
       <c r="C11" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>250</v>
       </c>
       <c r="B12" t="s">
-        <v>224</v>
+        <v>251</v>
       </c>
       <c r="C12" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>225</v>
+        <v>252</v>
       </c>
       <c r="B13" t="s">
-        <v>226</v>
+        <v>253</v>
       </c>
       <c r="C13" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>